<commit_message>
Seeds: state actualizado de días 27-30 abril + 1 mayo
State files que sembrarán el persistent disk en el primer arranque
de Render Starter:
- pedidos_dia/2026-04-27..30 con folios y ajustes vigentes
- pedidos_dia/2026-05-01 (nuevo día, 10 hospitales)
- extras_dia/2026-04-29 (folio 93 ALMACÉN EHMO) y 2026-05-01
- folio_counter actualizados (EHMO y comedores)
- Lista_Precios_EHMO.xlsx con cambios recientes

Excluye del seed (gitignore):
- data/*.backup_*.xlsx (respaldos de la lista de precios)
- storage/{pedidos,extras}_dia/_backups/ (recuperación local)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Lista_Precios_EHMO.xlsx
+++ b/data/Lista_Precios_EHMO.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ACELGAS</t>
+          <t>JUGO DE UVA 250 ML</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>24.5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -510,7 +510,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AGUACATE HASS</t>
+          <t>JUGO DE MANZANA 250 ML</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57.5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -528,7 +528,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AJO</t>
+          <t>DULCE DE AMARANTO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>77.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
@@ -546,7 +546,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ALMENDRA</t>
+          <t>PAN DULCE DONAS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>277.5</v>
+        <v>131.8</v>
       </c>
     </row>
     <row r="6">
@@ -564,7 +564,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>APIO</t>
+          <t>ACELGAS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="7">
@@ -582,7 +582,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AVENA INTEGRAL</t>
+          <t>AGUACATE HASS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>44.8</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="8">
@@ -600,7 +600,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BETABEL</t>
+          <t>AJO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>28.5</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="9">
@@ -618,7 +618,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BROCOLI</t>
+          <t>ALMENDRA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>24.5</v>
+        <v>277.5</v>
       </c>
     </row>
     <row r="10">
@@ -636,7 +636,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CACAHUATE TOSTADO</t>
+          <t>APIO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>97.5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -654,7 +654,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CALABACITA ITALIANA</t>
+          <t>AVENA INTEGRAL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24.5</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="12">
@@ -672,7 +672,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CALABAZA DE CASTILLA</t>
+          <t>BETABEL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>43.5</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="13">
@@ -690,7 +690,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CAMOTE AMARILLO</t>
+          <t>BROCOLI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -699,7 +699,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>97.5</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="14">
@@ -708,7 +708,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CANELA ENTERA</t>
+          <t>CACAHUATE TOSTADO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>494.5</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="15">
@@ -726,7 +726,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CEBOLLA BLANCA</t>
+          <t>CALABACITA ITALIANA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15.5</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="16">
@@ -744,7 +744,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CEBOLLA MORADA</t>
+          <t>CALABAZA DE CASTILLA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>17.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="17">
@@ -762,7 +762,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CHAMPIÑON</t>
+          <t>CAMOTE AMARILLO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>143.5</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="18">
@@ -780,7 +780,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CHAYOTE SIN ESPINA</t>
+          <t>CANELA ENTERA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>27.5</v>
+        <v>494.5</v>
       </c>
     </row>
     <row r="19">
@@ -798,7 +798,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CHICHARO LIMPIO</t>
+          <t>CEBOLLA BLANCA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>200.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="20">
@@ -816,7 +816,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CHILE ANCHO SECO</t>
+          <t>CEBOLLA MORADA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>187.5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="21">
@@ -834,7 +834,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CHILE ARBOL SECO</t>
+          <t>CHAMPIÑON</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>158.5</v>
+        <v>143.5</v>
       </c>
     </row>
     <row r="22">
@@ -852,7 +852,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CHILE CUARESMEÑO</t>
+          <t>CHAYOTE SIN ESPINA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>71.5</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="23">
@@ -870,7 +870,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CHILE GUAJILLO SECO</t>
+          <t>CHICHARO LIMPIO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>138.5</v>
+        <v>200.5</v>
       </c>
     </row>
     <row r="24">
@@ -888,7 +888,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CHILE HABANERO</t>
+          <t>CHILE ANCHO SECO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>114.5</v>
+        <v>187.5</v>
       </c>
     </row>
     <row r="25">
@@ -906,7 +906,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CHILE MORITA SECO</t>
+          <t>CHILE ARBOL SECO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>149.5</v>
+        <v>158.5</v>
       </c>
     </row>
     <row r="26">
@@ -924,7 +924,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CHILE MULATO</t>
+          <t>CHILE CUARESMEÑO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>265.5</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="27">
@@ -942,7 +942,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CHILE PASILLA SECO</t>
+          <t>CHILE GUAJILLO SECO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>285.5</v>
+        <v>138.5</v>
       </c>
     </row>
     <row r="28">
@@ -960,7 +960,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CHILE POBLANO PARA RELLENAR</t>
+          <t>CHILE HABANERO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>117.5</v>
+        <v>114.5</v>
       </c>
     </row>
     <row r="29">
@@ -978,7 +978,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CHILE SERRANO</t>
+          <t>CHILE MORITA SECO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>57.5</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="30">
@@ -996,7 +996,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CILANTRO</t>
+          <t>CHILE MULATO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>39.5</v>
+        <v>265.5</v>
       </c>
     </row>
     <row r="31">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CIRUELA PASA</t>
+          <t>CHILE PASILLA SECO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>171.5</v>
+        <v>285.5</v>
       </c>
     </row>
     <row r="32">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CIRUELA ROJA</t>
+          <t>CHILE POBLANO PARA RELLENAR</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>164.5</v>
+        <v>117.5</v>
       </c>
     </row>
     <row r="33">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COL BLANCA</t>
+          <t>CHILE SERRANO</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>39.5</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="34">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>COLIFLOR</t>
+          <t>CILANTRO</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>35.5</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="35">
@@ -1086,16 +1086,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>COMINO ENTERO 60G</t>
+          <t>CIRUELA PASA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>59.5</v>
+        <v>171.5</v>
       </c>
     </row>
     <row r="36">
@@ -1104,16 +1104,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>COMINO MOLIDO 60G</t>
+          <t>CIRUELA ROJA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>79.5</v>
+        <v>164.5</v>
       </c>
     </row>
     <row r="37">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DURAZNO AMARILLO</t>
+          <t>COL BLANCA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>149.5</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="38">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EJOTE</t>
+          <t>COLIFLOR</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>44.5</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="39">
@@ -1158,16 +1158,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ELOTE ENTERO</t>
+          <t>COMINO ENTERO 60G</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>58.5</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="40">
@@ -1176,16 +1176,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ELOTE PROCESADO CONGELADO</t>
+          <t>COMINO MOLIDO 60G</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>224.5</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="41">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EPAZOTE</t>
+          <t>DURAZNO AMARILLO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>32.5</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="42">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ESPINACAS</t>
+          <t>EJOTE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>39.5</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="43">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FLOR DE CALABAZA</t>
+          <t>ELOTE ENTERO</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>154.5</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="44">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>FLOR DE JAMAICA</t>
+          <t>ELOTE PROCESADO CONGELADO</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>149.5</v>
+        <v>224.5</v>
       </c>
     </row>
     <row r="45">
@@ -1266,16 +1266,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FORMULA DE INICIO NAN ETAPA 1 POLVO  400 G</t>
+          <t>EPAZOTE</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>306.6</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="46">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>FRIJOL BAYO</t>
+          <t>ESPINACAS</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>58.8</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="47">
@@ -1302,16 +1302,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GELATINA SIN AZUCAR</t>
+          <t>FLOR DE CALABAZA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>23.8</v>
+        <v>154.5</v>
       </c>
     </row>
     <row r="48">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GERMEN DE SOYA</t>
+          <t>FLOR DE JAMAICA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>80</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="49">
@@ -1338,16 +1338,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GUANABANA</t>
+          <t>FORMULA DE INICIO NAN ETAPA 1 POLVO  400 G</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>98.5</v>
+        <v>306.6</v>
       </c>
     </row>
     <row r="50">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GUAYABA</t>
+          <t>FRIJOL BAYO</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>42.5</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="51">
@@ -1374,16 +1374,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HIERBABUENA</t>
+          <t>GELATINA SIN AZUCAR</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>36.5</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="52">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HIERBAS DE OLOR</t>
+          <t>GERMEN DE SOYA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>124.5</v>
+        <v>80</v>
       </c>
     </row>
     <row r="53">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>HUEVO BLANCO</t>
+          <t>GUANABANA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>49.5</v>
+        <v>98.5</v>
       </c>
     </row>
     <row r="54">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JICAMA</t>
+          <t>GUAYABA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>17</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="55">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>JITOMATE BOLA</t>
+          <t>HIERBABUENA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>93.5</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="56">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JITOMATE SALADET</t>
+          <t>HIERBAS DE OLOR</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>57.5</v>
+        <v>124.5</v>
       </c>
     </row>
     <row r="57">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LECHUGA ITALIANA</t>
+          <t>HUEVO BLANCO</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>58.5</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="58">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LECHUGA OREJONA</t>
+          <t>JICAMA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>58.5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LECHUGA ROMANA</t>
+          <t>JITOMATE BOLA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>32</v>
+        <v>93.5</v>
       </c>
     </row>
     <row r="60">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LIMON AGRIO CON SEMILLA</t>
+          <t>JITOMATE SALADET</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>46.5</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="61">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LIMON SIN SEMILLA</t>
+          <t>LECHUGA ITALIANA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>46.5</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="62">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MAMEY</t>
+          <t>LECHUGA OREJONA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1581,7 +1581,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>78.5</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="63">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MANDARINA</t>
+          <t>LECHUGA ROMANA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>48.5</v>
+        <v>32</v>
       </c>
     </row>
     <row r="64">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MANGO ATAULFO</t>
+          <t>LIMON AGRIO CON SEMILLA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>149.5</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="65">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MANGO MANILA</t>
+          <t>LIMON SIN SEMILLA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>149.5</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="66">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MANZANA GOLDEN</t>
+          <t>MAMEY</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>76.5</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="67">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MELON CHINO</t>
+          <t>MANDARINA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>36.5</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="68">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MELON VALENCIANO</t>
+          <t>MANGO ATAULFO</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>29.5</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="69">
@@ -1698,16 +1698,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MERMELADA DE FRESA INDIVIDUAL 20 G CAJA 250 PZ</t>
+          <t>MANGO MANILA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CAJA</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>800</v>
+        <v>149.5</v>
       </c>
     </row>
     <row r="70">
@@ -1716,16 +1716,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MIEL DE ABEJA</t>
+          <t>MANZANA GOLDEN</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>128.8</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="71">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>NARANJA</t>
+          <t>MELON CHINO</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>25.5</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="72">
@@ -1752,16 +1752,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>NIEVE DE SABORES</t>
+          <t>MELON VALENCIANO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>91</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="73">
@@ -1770,16 +1770,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>NOPAL</t>
+          <t>MERMELADA DE FRESA INDIVIDUAL 20 G CAJA 250 PZ</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>CAJA</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>29.5</v>
+        <v>800</v>
       </c>
     </row>
     <row r="74">
@@ -1788,16 +1788,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>NOPAL SIN ESPINAS</t>
+          <t>MIEL DE ABEJA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>29.5</v>
+        <v>128.8</v>
       </c>
     </row>
     <row r="75">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>NUEZ LIMPIA EN MITADES</t>
+          <t>NARANJA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>364.5</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="76">
@@ -1824,16 +1824,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NUEZ LIMPIA ENTERA</t>
+          <t>NIEVE DE SABORES</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>364.5</v>
+        <v>91</v>
       </c>
     </row>
     <row r="77">
@@ -1842,16 +1842,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>OREGANO EN HOJA 60G</t>
+          <t>NOPAL</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>89.5</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="78">
@@ -1860,16 +1860,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PALANQUETA DE CACAHUATE 30 G</t>
+          <t>NOPAL SIN ESPINAS</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>50</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="79">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PAPA AMARILLA</t>
+          <t>NUEZ LIMPIA EN MITADES</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>40.5</v>
+        <v>364.5</v>
       </c>
     </row>
     <row r="80">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PAPA BLANCA</t>
+          <t>NUEZ LIMPIA ENTERA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>36.5</v>
+        <v>364.5</v>
       </c>
     </row>
     <row r="81">
@@ -1914,16 +1914,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PAPA CAMBRAY</t>
+          <t>OREGANO EN HOJA 60G</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>44.5</v>
+        <v>89.5</v>
       </c>
     </row>
     <row r="82">
@@ -1932,16 +1932,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PAPAYA MARADOL</t>
+          <t>PALANQUETA DE CACAHUATE 30 G</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>43.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="83">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PEPINO</t>
+          <t>PAPA AMARILLA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>54.5</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="84">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PERA MANTEQUILLA</t>
+          <t>PAPA BLANCA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>82.5</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="85">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PEREJIL</t>
+          <t>PAPA CAMBRAY</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>36.5</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="86">
@@ -2004,16 +2004,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PIMIENTA NEGRA ENTERA 60G</t>
+          <t>PAPAYA MARADOL</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>103.5</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="87">
@@ -2022,16 +2022,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PIMIENTA NEGRA MOLIDA 60G</t>
+          <t>PEPINO</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>103.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="88">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PIMIENTO MORRON</t>
+          <t>PERA MANTEQUILLA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>119.5</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="89">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PIMIENTO MORRON VERDE</t>
+          <t>PEREJIL</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>119.5</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="90">
@@ -2076,16 +2076,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PIÑA MIEL</t>
+          <t>PIMIENTA NEGRA ENTERA 60G</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>32.5</v>
+        <v>103.5</v>
       </c>
     </row>
     <row r="91">
@@ -2094,16 +2094,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PLATANO DOMINICO</t>
+          <t>PIMIENTA NEGRA MOLIDA 60G</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>89.5</v>
+        <v>103.5</v>
       </c>
     </row>
     <row r="92">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PLATANO MACHO</t>
+          <t>PIMIENTO MORRON</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2121,7 +2121,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>37.5</v>
+        <v>119.5</v>
       </c>
     </row>
     <row r="93">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PLATANO TABASCO</t>
+          <t>PIMIENTO MORRON VERDE</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>45</v>
+        <v>119.5</v>
       </c>
     </row>
     <row r="94">
@@ -2148,16 +2148,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>POLVO PARA HORNEAR 454 G</t>
+          <t>PIÑA MIEL</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>60</v>
+        <v>32.5</v>
       </c>
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="n"/>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>RABANO CHICO</t>
+          <t>PLATANO DOMINICO</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>30.5</v>
+        <v>89.5</v>
       </c>
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="n"/>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>REPOLLO</t>
+          <t>PLATANO MACHO</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>22</v>
+        <v>37.5</v>
       </c>
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="n"/>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SANDIA</t>
+          <t>PLATANO TABASCO</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>20.5</v>
+        <v>45</v>
       </c>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
@@ -2228,16 +2228,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TAMARINDO</t>
+          <t>POLVO PARA HORNEAR 454 G</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>134.5</v>
+        <v>60</v>
       </c>
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="n"/>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TE DE LIMON</t>
+          <t>RABANO CHICO</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>77.5</v>
+        <v>30.5</v>
       </c>
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="n"/>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TE DE MANZANILLA</t>
+          <t>REPOLLO</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>110.5</v>
+        <v>22</v>
       </c>
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="n"/>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TE DE YERBABUENA</t>
+          <t>SANDIA</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>36.5</v>
+        <v>20.5</v>
       </c>
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="n"/>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TOMATE VERDE LIMPIO</t>
+          <t>TAMARINDO</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>61.5</v>
+        <v>134.5</v>
       </c>
     </row>
     <row r="103">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TOMILLO</t>
+          <t>TE DE LIMON</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>177.5</v>
+        <v>77.5</v>
       </c>
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="n"/>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>TUNA VERDE</t>
+          <t>TE DE MANZANILLA</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2355,7 +2355,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>35</v>
+        <v>110.5</v>
       </c>
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="n"/>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>UVA PASA DESHIDRATADA</t>
+          <t>TE DE YERBABUENA</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>137.5</v>
+        <v>36.5</v>
       </c>
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="n"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>UVA VERDE SIN SEMILLA</t>
+          <t>TOMATE VERDE LIMPIO</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2395,7 +2395,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>127.5</v>
+        <v>61.5</v>
       </c>
       <c r="I106" s="3" t="n"/>
     </row>
@@ -2405,15 +2405,87 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>TOMILLO</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>177.5</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>TUNA VERDE</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>UVA PASA DESHIDRATADA</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>UVA VERDE SIN SEMILLA</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>127.5</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
           <t>ZANAHORIA</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="D107" t="n">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
         <v>16.5</v>
       </c>
     </row>

</xml_diff>